<commit_message>
docs: update Swagger annotations with frontend references and remove unused ServiceImpl
</commit_message>
<xml_diff>
--- a/folder_template/Template1_Project Tracking.xlsx
+++ b/folder_template/Template1_Project Tracking.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11880"/>
+    <workbookView windowWidth="19200" windowHeight="8000"/>
   </bookViews>
   <sheets>
     <sheet name="Project" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Project!$A$3:$E$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Project!$A$3:$E$20</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="107">
   <si>
     <t>Total Project Tracking</t>
   </si>
@@ -137,87 +137,90 @@
     <t>Simple</t>
   </si>
   <si>
+    <t>Đỗ Quốc Huy</t>
+  </si>
+  <si>
+    <t>Jockey Management</t>
+  </si>
+  <si>
+    <t>Jockey Data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manages information and profiles for jockeys. Updates their status and assigns them to upcoming races.	</t>
+  </si>
+  <si>
+    <t>Bùi Đức Tài</t>
+  </si>
+  <si>
+    <t>Created Jockey.tsx dashboard, implemented mounts registration status check, and integrated kqp-based rule violations table.</t>
+  </si>
+  <si>
+    <t>Manage Race &amp; Tournaments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Race Management	</t>
+  </si>
+  <si>
+    <t>Creates new seasons and races, schedules events, and allocates horses and jockeys to specific races.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Complex  </t>
+  </si>
+  <si>
+    <t>Resolved the logic to prevent race scheduling conflicts, implemented season class rules configuration, and hid budget/purse inputs.</t>
+  </si>
+  <si>
+    <t>View Public Schedules &amp; Results</t>
+  </si>
+  <si>
+    <t>Public Data</t>
+  </si>
+  <si>
+    <t>Guest, All Users</t>
+  </si>
+  <si>
+    <t>Allows guests to view upcoming race schedules and past race results without requiring an account login.</t>
+  </si>
+  <si>
+    <t>Cao Nhật Lâm, Bùi Đức Tài, Võ Thành Đạt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done	</t>
+  </si>
+  <si>
+    <t>Designed Landing.tsx homepage, integrated live countdown timer for upcoming meetings, and implemented public race results table view.</t>
+  </si>
+  <si>
+    <t>Referee Actions</t>
+  </si>
+  <si>
+    <t>Race Execution</t>
+  </si>
+  <si>
+    <t>Referee</t>
+  </si>
+  <si>
+    <t>Dedicated functionality for referees to update match statuses, input final results, and record placements after a race ends.</t>
+  </si>
+  <si>
+    <t>Implemented RefereeHub.tsx, designed forms to log rule violations during active races, and set up backend RefereeService mappings.</t>
+  </si>
+  <si>
+    <t>Public Chat</t>
+  </si>
+  <si>
+    <t>Communication</t>
+  </si>
+  <si>
+    <t>All Users</t>
+  </si>
+  <si>
+    <t>A general chat channel that allows users to discuss races and tournaments.</t>
+  </si>
+  <si>
     <t>Cao Nhật Lâm, Đỗ Quốc Huy</t>
   </si>
   <si>
-    <t>Jockey Management</t>
-  </si>
-  <si>
-    <t>Jockey Data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manages information and profiles for jockeys. Updates their status and assigns them to upcoming races.	</t>
-  </si>
-  <si>
-    <t>Bùi Đức Tài</t>
-  </si>
-  <si>
-    <t>Created Jockey.tsx dashboard, implemented mounts registration status check, and integrated kqp-based rule violations table.</t>
-  </si>
-  <si>
-    <t>Manage Race &amp; Tournaments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Race Management	</t>
-  </si>
-  <si>
-    <t>Creates new seasons and races, schedules events, and allocates horses and jockeys to specific races.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Complex  </t>
-  </si>
-  <si>
-    <t>Resolved the logic to prevent race scheduling conflicts, implemented season class rules configuration, and hid budget/purse inputs.</t>
-  </si>
-  <si>
-    <t>View Public Schedules &amp; Results</t>
-  </si>
-  <si>
-    <t>Public Data</t>
-  </si>
-  <si>
-    <t>Guest, All Users</t>
-  </si>
-  <si>
-    <t>Allows guests to view upcoming race schedules and past race results without requiring an account login.</t>
-  </si>
-  <si>
-    <t>Cao Nhật Lâm, Bùi Đức Tài, Võ Thành Đạt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Done	</t>
-  </si>
-  <si>
-    <t>Designed Landing.tsx homepage, integrated live countdown timer for upcoming meetings, and implemented public race results table view.</t>
-  </si>
-  <si>
-    <t>Referee Actions</t>
-  </si>
-  <si>
-    <t>Race Execution</t>
-  </si>
-  <si>
-    <t>Referee</t>
-  </si>
-  <si>
-    <t>Dedicated functionality for referees to update match statuses, input final results, and record placements after a race ends.</t>
-  </si>
-  <si>
-    <t>Implemented RefereeHub.tsx, designed forms to log rule violations during active races, and set up backend RefereeService mappings.</t>
-  </si>
-  <si>
-    <t>Public Chat</t>
-  </si>
-  <si>
-    <t>Communication</t>
-  </si>
-  <si>
-    <t>All Users</t>
-  </si>
-  <si>
-    <t>A general chat channel that allows users to discuss races and tournaments.</t>
-  </si>
-  <si>
     <t>May need to consider WebSocket integration in the future for real-time updates.</t>
   </si>
   <si>
@@ -248,7 +251,7 @@
     <t>Provides interactive SVG/CSS performance charts and historical statistics on the spectator dashboard.</t>
   </si>
   <si>
-    <t>Cao Nhật Lâm, Đỗ Quốc Huy, Võ Thành Đạt</t>
+    <t>Đỗ Quốc Huy, Võ Thành Đạt</t>
   </si>
   <si>
     <t>Designed responsive SVG bar/line charts and performance summary tables with mobile layout support.</t>
@@ -284,7 +287,7 @@
     <t>Implements backend page requests and frontend search input filters for listing users, horses, and races.</t>
   </si>
   <si>
-    <t>Cao Nhật Lâm, Bùi Đức Tài, Lê Nguyễn Chánh Nghĩa</t>
+    <t>Lê Nguyễn Chánh Nghĩa, Đỗ Quốc Huy,Võ Thành Đạt</t>
   </si>
   <si>
     <t>Optimized database loading times and improved UI usability with server-side pagination controllers.</t>
@@ -344,7 +347,7 @@
     <t>Establishing consistent UI components, color palettes, and global layout styles.</t>
   </si>
   <si>
-    <t>Võ Thành Đạt, Đỗ Đức Huy</t>
+    <t>Võ Thành Đạt, Đỗ Quốc Huy</t>
   </si>
   <si>
     <t>Implemented design system with shared component library for consistent branding.</t>
@@ -1023,7 +1026,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1082,17 +1085,20 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1362,18 +1368,18 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:I20"/>
-  <sheetFormatPr defaultColWidth="10.7809523809524" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="10.7818181818182" defaultRowHeight="12.5"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
-    <col min="2" max="2" width="35.3238095238095" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13.6666666666667" style="2" customWidth="1"/>
+    <col min="2" max="2" width="35.3272727272727" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.6636363636364" style="2" customWidth="1"/>
     <col min="4" max="4" width="14" style="2" customWidth="1"/>
-    <col min="5" max="5" width="50.6666666666667" style="2" customWidth="1"/>
-    <col min="6" max="6" width="11.1047619047619" style="2" customWidth="1"/>
-    <col min="7" max="7" width="19.7904761904762" style="2" customWidth="1"/>
-    <col min="8" max="8" width="7.78095238095238" style="2" customWidth="1"/>
-    <col min="9" max="9" width="45.447619047619" style="2" customWidth="1"/>
-    <col min="10" max="16384" width="10.7809523809524" style="2" customWidth="1"/>
+    <col min="5" max="5" width="50.6636363636364" style="2" customWidth="1"/>
+    <col min="6" max="6" width="11.1090909090909" style="2" customWidth="1"/>
+    <col min="7" max="7" width="19.7909090909091" style="2" customWidth="1"/>
+    <col min="8" max="8" width="7.78181818181818" style="2" customWidth="1"/>
+    <col min="9" max="9" width="45.4454545454545" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="10.7818181818182" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.4" customHeight="1" spans="1:9">
@@ -1519,7 +1525,7 @@
       <c r="D7" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="24" t="s">
+      <c r="E7" s="25" t="s">
         <v>33</v>
       </c>
       <c r="F7" s="8" t="s">
@@ -1669,13 +1675,13 @@
         <v>34</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="H12" s="12" t="s">
         <v>51</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" ht="37.5" customHeight="1" spans="1:9">
@@ -1684,28 +1690,28 @@
         <v>10</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D13" s="10" t="s">
         <v>48</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>23</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H13" s="12" t="s">
         <v>17</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" ht="37.5" customHeight="1" spans="1:9">
@@ -1714,28 +1720,28 @@
         <v>11</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F14" s="16" t="s">
         <v>15</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H14" s="19" t="s">
         <v>17</v>
       </c>
       <c r="I14" s="17" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" ht="37.5" customHeight="1" spans="1:9">
@@ -1744,28 +1750,28 @@
         <v>12</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F15" s="16" t="s">
         <v>23</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H15" s="19" t="s">
         <v>17</v>
       </c>
       <c r="I15" s="17" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" ht="37.5" customHeight="1" spans="1:9">
@@ -1774,28 +1780,28 @@
         <v>13</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F16" s="16" t="s">
         <v>15</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H16" s="19" t="s">
         <v>17</v>
       </c>
       <c r="I16" s="17" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" ht="25" customHeight="1" spans="1:9">
@@ -1804,28 +1810,28 @@
         <v>14</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F17" s="16" t="s">
         <v>15</v>
       </c>
       <c r="G17" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H17" s="19" t="s">
         <v>17</v>
       </c>
       <c r="I17" s="17" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18" ht="25" customHeight="1" spans="1:9">
@@ -1834,28 +1840,28 @@
         <v>15</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F18" s="16" t="s">
         <v>15</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="H18" s="19" t="s">
         <v>17</v>
       </c>
       <c r="I18" s="17" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="19" ht="47" customHeight="1" spans="1:9">
@@ -1864,62 +1870,62 @@
         <v>16</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D19" s="18" t="s">
         <v>60</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F19" s="16" t="s">
         <v>15</v>
       </c>
       <c r="G19" s="18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H19" s="19" t="s">
         <v>17</v>
       </c>
       <c r="I19" s="17" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
-    <row r="20" ht="25.5" spans="1:9">
+    <row r="20" ht="25" spans="1:9">
       <c r="A20" s="16">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D20" s="18" t="s">
         <v>60</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F20" s="16" t="s">
         <v>15</v>
       </c>
       <c r="G20" s="23" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H20" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="I20" s="22" t="s">
-        <v>105</v>
+      <c r="I20" s="24" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A3:E19" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A3:E20" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <dataValidations count="2">

</xml_diff>